<commit_message>
Updated the RTM notebook to include the new components
Updated the RTM notebook to include the new names of components and added my input to the AI register.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>UI.Requester.SubmitRequestForm -&gt; POST /requests -&gt; RequestService -&gt; RequestRepository</t>
+          <t>Pages/Requests/Submit.cshtml (SubmitModel) -&gt; POST /api/v1/requests -&gt; RequestService -&gt; RequestRepository</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Category selector -&gt; GET /categories -&gt; CategoryService -&gt; CategoryRepository</t>
+          <t>_CategorySelect partial on the submit page -&gt; GET /api/v1/categories -&gt; CategoryService -&gt; CategoryRepository</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>UI.Requester.RequestStatusView -&gt; GET /requests/{id}</t>
+          <t>Pages/Requests/Details.cshtml (DetailsModel) with the status badge tag helper -&gt; GET /api/v1/requests/{id}</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>UI.Requester.RequestHistoryView -&gt; GET /requests?mine -&gt; AuthorisationPolicy</t>
+          <t>Pages/Requests/Index.cshtml (IndexModel) -&gt; GET /api/v1/requests in own scope -&gt; AuthorisationPolicy</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>RequestHistoryView filters -&gt; GET /requests?status=</t>
+          <t>_FilterBar partial on Pages/Requests/Index.cshtml -&gt; GET /api/v1/requests with status filter</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>StatusTransitionService -&gt; FeedbackService -&gt; GET /feedback -&gt; UI.Requester.FeedbackPanel</t>
+          <t>StatusTransitionService -&gt; FeedbackService -&gt; GET /api/v1/feedback -&gt; _FeedbackList partial on Pages/Requests/Index.cshtml</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>UI.Staff.QueueView -&gt; GET /requests/queue -&gt; AuthorisationPolicy -&gt; RequestRepository</t>
+          <t>Pages/Staff/Queue.cshtml (QueueModel) with StaffQueueViewComponent -&gt; GET /api/v1/requests/queue -&gt; AuthorisationPolicy -&gt; RequestRepository</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>QueueView filter and sort controls -&gt; API query parameters</t>
+          <t>_FilterBar partial inside StaffQueueViewComponent -&gt; GET /api/v1/requests query parameters</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>UI.Staff.RequestDetailView -&gt; GET /requests/{id} -&gt; AuthorisationPolicy</t>
+          <t>Pages/Staff/Details.cshtml (DetailsModel) with _RequestDetail and _HistoryList partials -&gt; GET /api/v1/requests/{id} -&gt; AuthorisationPolicy</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>UI.Staff.ActionPanel -&gt; POST /requests/{id}/assignment -&gt; AssignmentService -&gt; RequestRepository</t>
+          <t>Pages/Staff/Details.cshtml OnPostAcceptAsync -&gt; POST /api/v1/requests/{id}/assignment -&gt; AssignmentService -&gt; RequestRepository</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>ActionPanel -&gt; PATCH /requests/{id}/status -&gt; StatusTransitionService</t>
+          <t>Pages/Staff/Details.cshtml OnPostTransitionAsync -&gt; PATCH /api/v1/requests/{id}/status -&gt; StatusTransitionService</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>ActionPanel -&gt; POST /requests/{id}/notes -&gt; HistoryRepository</t>
+          <t>Pages/Staff/Details.cshtml OnPostAddNoteAsync -&gt; POST /api/v1/requests/{id}/notes -&gt; HistoryRepository</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>ActionPanel -&gt; PATCH /status -&gt; AuthorisationPolicy + StatusTransitionService + FeedbackService</t>
+          <t>Pages/Staff/Details.cshtml OnPostCloseAsync -&gt; PATCH /api/v1/requests/{id}/status -&gt; AuthorisationPolicy, StatusTransitionService and FeedbackService</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>UI.Management.OversightDashboard -&gt; GET /reports/overview -&gt; ReportingService</t>
+          <t>Pages/Management/Oversight.cshtml with OversightTotalsViewComponent -&gt; GET /api/v1/reports/overview -&gt; ReportingService</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>OversightDashboard lifecycle filters -&gt; ReportingService</t>
+          <t>Pages/Management/Oversight.cshtml lifecycle filters -&gt; ReportingService</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>OversightDashboard grouping -&gt; ReportingService</t>
+          <t>OversightTotalsViewComponent grouping -&gt; ReportingService</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>UI.Management.ReportView -&gt; GET /reports/performance -&gt; ReportingService</t>
+          <t>Pages/Management/Reports.cshtml (ReportsModel) -&gt; GET /api/v1/reports/performance -&gt; ReportingService</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>UI.Admin.UserAdminView -&gt; /admin/users -&gt; UserRoleService</t>
+          <t>Pages/Admin/Users.cshtml (UsersModel) -&gt; /api/v1/admin/users -&gt; UserRoleService</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>UI.Admin.RoleAdminView -&gt; /admin/roles -&gt; AuthorisationPolicy (single decision point)</t>
+          <t>Pages/Admin/Roles.cshtml (RolesModel) -&gt; /api/v1/admin/roles -&gt; AuthorisationPolicy as the single decision point</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>UI.Admin.CategoryAdminView -&gt; /admin/categories -&gt; CategoryService</t>
+          <t>Pages/Admin/Categories.cshtml (CategoriesModel) -&gt; /api/v1/admin/categories -&gt; CategoryService</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>UI.Admin audit view -&gt; /admin/audit -&gt; AuditService</t>
+          <t>Pages/Admin/Audit.cshtml (AuditModel) -&gt; /api/v1/admin/audit -&gt; AuditService</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Reuse UI.Management.ReportView at summary scope (access model pending CR-007)</t>
+          <t>Reuse Pages/Management/Reports.cshtml at summary scope (access model pending CR-007)</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>UI.Requester submission flow (single guided form)</t>
+          <t>Pages/Requests/Submit.cshtml, one guided form with validation messages for each field</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>FeedbackService write + UI.Requester refresh path</t>
+          <t>FeedbackService write; JavaScript fetch polling refreshes the status partial on Pages/Requests/Details.cshtml</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>AuthorisationPolicy + ownership-scoped repository queries</t>
+          <t>AuthorisationPolicy with ownership scoped repository queries in every page model</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Queue and oversight query paths (RequestRepository, ReportingService)</t>
+          <t>Queue and oversight query paths: StaffQueueViewComponent, RequestRepository, ReportingService</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>AssignmentService + StatusTransitionService behind the API boundary</t>
+          <t>AssignmentService and StatusTransitionService behind the API boundary</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>AuthorisationPolicy as the single authorisation decision point</t>
+          <t>AuthorisationPolicy invoked by every page handler and every endpoint</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>AuditService and append-only history writes on every controlled action</t>
+          <t>AuditService and append only history writes on every controlled action</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
@@ -3678,8 +3678,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="9" t="n"/>
     </row>
@@ -3828,8 +3826,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -4013,8 +4009,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="n"/>
     </row>

</xml_diff>

<commit_message>
closed off gaps in the rtm, and updated UI
closed off gaps in the rtm, and updated UI file so interfaces match.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
@@ -670,7 +670,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages and Web API (.NET 10 LTS, C# 13); PostgreSQL 17.x (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -680,17 +680,17 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: branch feature/fr-001-submit; migration 001_request</t>
+          <t>Core/Services/RequestService.SubmitAsync; Data/Migrations/001_request.sql; Pages/Requests/Submit.cshtml</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-001.1 valid submit; TC-001.2 missing field blocked</t>
+          <t>RequestServiceTests (Overlong_title_is_refused, Staff_cannot_submit_requests_without_the_permission); not yet executed</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x reference table; ASP.NET Core (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -767,17 +767,17 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: seed migration 002_category</t>
+          <t>Core/Services/CategoryService; Data/Migrations/002_category.sql; category select on Pages/Requests/Submit.cshtml</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-002.1 controlled values only; TC-002.2 empty category blocked</t>
+          <t>Covered indirectly by RequestServiceTests; page test planned</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages; JavaScript fetch polling for status (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -854,17 +854,17 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>UI branch</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>Core/Services/RequestService.GetAsync; Pages/Requests/Details.cshtml; TagHelpers/StatusBadgeTagHelper</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-003.1 plain-language status; TC-003.2 no status control rendered</t>
+          <t>StatusRulesTests (Display_text_is_plain_language); page test for AC-003.2 planned</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages; PostgreSQL 17.x (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -941,17 +941,17 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>RequestService.ListOwnAsync; Pages/Requests/Index.cshtml; index ix_request_requester</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-004.1 own requests only; TC-004.2 negative cross-requester access</t>
+          <t>RequestServiceTests scope cases; negative access test planned</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages; PostgreSQL 17.x indexes (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1028,17 +1028,17 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>UI branch</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Status filter on Pages/Requests/Index.cshtml; ListOwnAsync paging</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Planned: filter and empty state page test</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>In application only, JavaScript fetch polling; no email or SMS (ADR-003; conflict C-4)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -1202,17 +1202,17 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: raised by the FR-012 path</t>
+          <t>Core/Services/FeedbackService; Data/Migrations/004_feedback.sql; FeedbackController. No requester screen yet</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-007.1 visible within 15 s; TC-007.2 rejection reason present</t>
+          <t>NoteAndFeedbackTests (Nobody_can_mark_someone_elses_feedback_as_read); timing check planned</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages; policy based authorisation (ADR-003, ADR-005)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1289,17 +1289,17 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>RequestService.QueueAsync; Pages/Staff/Queue.cshtml; index ix_request_queue</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-008.1 authorised rows only; TC-008.2 unauthorised row absent</t>
+          <t>RequestServiceTests (The_queue_is_closed_to_requesters); not yet executed</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core; PostgreSQL 17.x indexes (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -1376,17 +1376,17 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Sort whitelist in RequestService.QueueAsync and RequestRepository; status filter on the queue page</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Planned: sort and filter tests</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q11" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages; policy based authorisation (ADR-003, ADR-005)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1463,17 +1463,17 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>RequestService.GetAsync with history and notes; Pages/Staff/Details.cshtml; _RequestFields and _HistoryList</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-010.1 full detail including action history</t>
+          <t>RequestServiceTests visibility cases; not yet executed</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x transactional conditional update through an ASP.NET Core service (ADR-002, ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1550,17 +1550,17 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: branch feature/fr-011-assign-accept; AssignmentService; migration 003_assignment</t>
+          <t>AssignmentService.AcceptAsync; RequestRepository.TryAssignAsync conditional update; Migrations/003_assignment.sql; Pages/Staff/Details.cshtml OnPostAcceptAsync</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-011.1 accept records owner + timestamp; TC-011.2 concurrent accept (N parallel, 1 succeeds)</t>
+          <t>RealDatabaseTests.Ten_staff_accepting_at_once_leaves_exactly_one_owner (TC-011.2) and AssignmentServiceTests; needs a test database, not yet executed</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>Baselined - M2 trace requirement</t>
+          <t>In Development - M2 trace requirement</t>
         </is>
       </c>
       <c r="Q13" s="5" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x transaction; ASP.NET Core service (ADR-002, ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -1637,17 +1637,17 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>StatusTransitionService.TransitionAsync; Core/Rules/StatusRules; Pages/Staff/Details.cshtml OnPostTransitionAsync</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-012.1 valid transition recorded; TC-012.2 invalid transition blocked</t>
+          <t>StatusTransitionServiceTests (7 cases) and StatusRulesTests; not yet executed</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x append only tables (ADR-002, ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -1724,17 +1724,17 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>Core/Services/NoteService; request_note table with an append only trigger. No screen yet</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-013.1 note saved with author + timestamp; no delete endpoint</t>
+          <t>NoteAndFeedbackTests (Only_the_owner_can_add_notes, An_empty_note_is_refused)</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="P15" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q15" s="5" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core policy based authorisation; PostgreSQL 17.x transaction (ADR-003, ADR-005)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -1811,17 +1811,17 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>TransitionAsync with the close permission; offered through NextStatuses on the staff page</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>StatusTransitionServiceTests close cases; not yet executed</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x aggregate queries; ASP.NET Core Razor Pages (ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x; schema addition pending CR-005 (ADR-003)</t>
+          <t>PostgreSQL 17.x; target response column not added (CR-005)</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x grouping with supporting indexes (ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core; PostgreSQL 17.x (ADR-003); export tooling pending CR-006</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core identity mechanism pending CR-003; PostgreSQL 17.x (ADR-003, ADR-005)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -2246,19 +2246,19 @@
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
+          <t>Backend branch</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>app_user table with is_active in Migrations/001_request.sql; Data/UserRepository. No admin screen</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
+        <is>
           <t>at M3</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
-      <c r="N21" s="6" t="inlineStr">
-        <is>
-          <t>at M3</t>
-        </is>
-      </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
           <t>at M4</t>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="P21" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q21" s="5" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core policy based authorisation; PostgreSQL 17.x role tables (ADR-003, ADR-005)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2333,17 +2333,17 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: enforcement path (admin UI later)</t>
+          <t>Migrations/005_rbac.sql (role, permission, role_permission, user_role) with the seeded matrix; Core/Rules/AuthorisationPolicy</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-020.1 role grants match actions; TC-020.2 non-administrator blocked</t>
+          <t>RequestServiceTests and AssignmentServiceTests permission cases (A_requester_cannot_accept_requests, A_requester_cannot_change_status)</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x reference data; ASP.NET Core (ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="M23" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Category table supports retire; no admin screen</t>
         </is>
       </c>
       <c r="N23" s="6" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x append only tables (ADR-002, ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -2507,17 +2507,17 @@
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Write path begins in Slice 1; read view -&gt; M3</t>
+          <t>request_status_history and request_note with block_history_changes triggers. Admin view not built</t>
         </is>
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>RealDatabaseTests.History_rows_cannot_be_changed_or_deleted</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages at summary scope (ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core Razor Pages, one guided form (ADR-003)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -2681,17 +2681,17 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>UI branch</t>
         </is>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: requester UI</t>
+          <t>One guided form on Pages/Requests/Submit.cshtml with a message against each field</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-N001 moderated walkthrough, 3 first-time users</t>
+          <t>Planned: moderated walkthrough with three first time users</t>
         </is>
       </c>
       <c r="O26" s="6" t="inlineStr">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>JavaScript fetch polling on Razor Pages; no push infrastructure (ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -2768,17 +2768,17 @@
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>Feedback written in the same transaction as the status change (FeedbackService). No refresh on the requester screen yet</t>
         </is>
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-N002 timed observation after an FR-012 transition</t>
+          <t>Planned: timed observation after a transition</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core policy based authorisation; ownership scoped queries (ADR-003, ADR-005)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -2855,17 +2855,17 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>AuthorisationPolicy.CanSee; scoped queries in RequestRepository; requester pages load own rows only</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-N003 negative access test using a direct reference ID</t>
+          <t>RequestServiceTests visibility cases; direct reference negative test planned</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x on Neon free plan; measured on Render free tier (ADR-003, ADR-007)</t>
+          <t>PostgreSQL 17.x indexes; measured on the Render and Neon free plans (ADR-007)</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -2942,17 +2942,17 @@
       </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
-          <t>Seed script for 1,000 requests - planned</t>
+          <t>Indexes ix_request_queue, ix_request_requester, ix_request_created in place. db/dev_seed.sql seeds a small set only</t>
         </is>
       </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Planned: TC-N004 timed load against the seeded dataset</t>
+          <t>Planned: timed load at 1,000 seeded requests</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x transactions; Read Committed with conditional update (ADR-002, ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3029,17 +3029,17 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>RequestRepository.TryAssignAsync and TryChangeStatusAsync guarded updates; version column; ck_request_owner_pair and ck_request_owner_vs_status</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-011.2 concurrent accept; TC-N005 lost-update test</t>
+          <t>RealDatabaseTests.Ten_staff_accepting_at_once_leaves_exactly_one_owner and The_database_itself_refuses_an_owner_on_a_Received_request</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>Baselined - M2 trace requirement</t>
+          <t>In Development - M2 trace requirement</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>ASP.NET Core authorisation policies (ADR-003, ADR-005)</t>
+          <t>Razor Pages; ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -3116,17 +3116,17 @@
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend and UI branches</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned</t>
+          <t>AuthorisationPolicy.Require called by every service; capabilities on the pages come from the same permissions (UI/CapabilityFactory)</t>
         </is>
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-N006 role matrix negative tests per endpoint</t>
+          <t>Permission refusal cases across the service tests; role matrix test planned</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x append only tables (ADR-002, ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -3203,17 +3203,17 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>Planned (M2)</t>
+          <t>Backend branch</t>
         </is>
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: history writes</t>
+          <t>Append only history and notes enforced by the block_history_changes triggers, not only by the application</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>Slice 1 - planned: TC-N007 entry present per action; alteration attempt fails</t>
+          <t>RealDatabaseTests.History_rows_cannot_be_changed_or_deleted</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>Baselined</t>
+          <t>In Development</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>PostgreSQL 17.x aggregates from the source tables, no separate store (ADR-001, ADR-003)</t>
+          <t>ASP.NET Core on .NET 10 (C# 13); Npgsql with SQL migrations; PostgreSQL 17.x (ADR-003)</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="M33" s="6" t="inlineStr">
         <is>
-          <t>at M3</t>
+          <t>Reporting reads the same tables; no reporting screen yet</t>
         </is>
       </c>
       <c r="N33" s="6" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Render free tier container; Neon free plan PostgreSQL 17.x (ADR-003, ADR-007)</t>
+          <t>Render free tier and Neon free plan (ADR-007)</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -3382,12 +3382,12 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>Hosting spike - planned</t>
+          <t>Not deployed yet; plan limits recorded in ADR-007</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>Planned: TC-N009 cost sheet checked against tier limits</t>
+          <t>Planned: cost sheet against the plan limits</t>
         </is>
       </c>
       <c r="O34" s="6" t="inlineStr">

</xml_diff>

<commit_message>
M2 rework: microservices requirements, ASRs, change control and ADR-004 revision 2
- PED v3: conflict C-5, NFR-010 growth readiness, open item statuses, ASR section, change register (CR-009 to CR-011, EC-001), Engineering Decisions and Comparisons section with the ADR-004 comparison tables
- ADR-004 revision 2: one web frontend service (option C) with P3 page composition, weighted comparison tables
- ASR register: ASR-05 restated, ASR-07 added, consequences rewritten for services
- RTM workbook: NFR-010 row, CR-009 to CR-011 and EC-001, ASR-07

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASR &amp; ADR Index" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RTM'!$A$2:$Q$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RTM'!$A$2:$Q$35</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3406,8 +3406,95 @@
         </is>
       </c>
     </row>
+    <row r="35" ht="25.5" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>NFR-010</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Growth readiness: able to expand in future without a redesign (added through CR-011).</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>ST-5</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Scale-out, data ownership and extension checks all pass (NFR-010)</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>ASR-07</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Pending revised ADR-001 (CR-010)</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Each service owns its data store; pending revised ADR-001/ADR-002 (CR-010)</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>ADR-004 revision 2: one web frontend service with no in-memory session state</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Pending revised ADR-001 (CR-010)</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>CR-010; CR-011; ADR-001; ADR-004</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>at M3</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>Planned: FR-011 concurrent-accept check against two copies of the owning service</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="inlineStr">
+        <is>
+          <t>at M4</t>
+        </is>
+      </c>
+      <c r="P35" s="5" t="inlineStr">
+        <is>
+          <t>Candidate (CR-011)</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>M. Malope</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:Q34"/>
+  <autoFilter ref="A2:Q35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3418,7 +3505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3678,8 +3765,113 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>CR-009</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>FR-007 (AC-007.2), FR-012 (AC-012.1)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Introduce Rejected as a terminal status that can only be reached from Received and always carries a reason.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>K. Marota proposes, M. Malope records</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CR-010</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>ADR-001 (to be superseded); Initial Architecture Strategy; RTM architecture and data columns; ADR-002, ADR-004 to ADR-007</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Move from the layered modular monolith (ADR-001) to microservices so the system can expand in future without a redesign. Functional scope stays the same.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Open; revised ADR-001 pending</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>K. Marota (architecture), M. Malope (requirements impact)</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CR-011</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>NFR-010 (new), ASR-05 (restated), ASR-07 (new), conflict C-5 (new)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Introduce NFR-010 Growth Readiness with three checks and no volume target; restate ASR-05; add ASR-07 and C-5.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>M. Malope</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>EC-001</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>FR-021 (AC-021.1)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Editorial correction: AC-021.1 cited AC-002.3, which does not exist; it now cites AC-002.1. No change in meaning.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>M. Malope</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3703,7 +3895,7 @@
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>ASR register (PED v2.0 section 5.2)</t>
+          <t>ASR register (PED v3.0, ASR section)</t>
         </is>
       </c>
     </row>
@@ -3800,12 +3992,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Cost and complexity sustainability</t>
+          <t>Cost and complexity sustainability while staying ready to grow (restated, CR-011)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>NFR-009; conflict C-4; RSK-003; RSK-014; RSK-016</t>
+          <t>NFR-009; conflicts C-4 and C-5; RSK-003; RSK-014; RSK-016</t>
         </is>
       </c>
     </row>
@@ -3826,6 +4018,23 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>ASR-07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Growth readiness (new, CR-011)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>NFR-010; conflict C-5; CR-010; CR-011</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -3873,7 +4082,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Proposed, awaiting approval</t>
+          <t>Proposed, awaiting approval; to be revised under CR-010</t>
         </is>
       </c>
     </row>
@@ -3939,7 +4148,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Proposed, awaiting approval</t>
+          <t>Proposed; revision 2 (08/10/2026) awaiting approval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align CR-010, ASR-04 and NFR-010 with ADR-001; split RTM workbook
Updates CR-010, ASR-04 and NFR-010 to match the approved ADR-001 service split (four services behind one API entry point, a schema per service in one PostgreSQL instance), so NFR-008 now stands unchanged. Splits the RTM workbook into separate RTM, change register and ASR/ADR index workbooks, following the new one-tab-per-workbook rule.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
@@ -7,8 +7,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RTM" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Register" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASR &amp; ADR Index" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RTM'!$A$2:$Q$35</definedName>
@@ -3497,731 +3495,4 @@
   <autoFilter ref="A2:Q35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Controlled changes raised against the M1 baseline</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>CR ID</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Affects</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Requested change</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>CR-001</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>NFR-002</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Confirm feedback latency as 15 s; correct the M1 'Z sec' wording.</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>CR-002</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>NFR-004</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Confirm 3 s at 1,000 seeded requests; record the seeding method.</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>CR-003</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>NFR-006, FR-020, D-004</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Close the authentication and authorisation decision.</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>G. Enright</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CR-004</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>FR-011 (AC-011.2)</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Confirm reassignment rules for an already-owned request.</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope with ST-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CR-005</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>FR-016 (AC-016.2)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Add a target-response field so 'overdue' is definable.</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope raises, K. Marota implements</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>CR-006</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>FR-018 (AC-018.2)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Decide whether reporting export is in scope or deferred.</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope with ST-3 and ST-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CR-007</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>FR-023</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Confirm sponsor view: dedicated or reuse management reporting.</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope with ST-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>CR-008</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>FR-002, FR-021</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Confirm the initial controlled category list content.</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope with ST-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>CR-009</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>FR-007 (AC-007.2), FR-012 (AC-012.1)</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Introduce Rejected as a terminal status that can only be reached from Received and always carries a reason.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>K. Marota proposes, M. Malope records</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>CR-010</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>ADR-001 (to be superseded); Initial Architecture Strategy; RTM architecture and data columns; ADR-002, ADR-004 to ADR-007</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Move from the layered modular monolith (ADR-001) to microservices so the system can expand in future without a redesign. Functional scope stays the same.</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Open; revised ADR-001 pending</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>K. Marota (architecture), M. Malope (requirements impact)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>CR-011</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>NFR-010 (new), ASR-05 (restated), ASR-07 (new), conflict C-5 (new)</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Introduce NFR-010 Growth Readiness with three checks and no volume target; restate ASR-05; add ASR-07 and C-5.</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>EC-001</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>FR-021 (AC-021.1)</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Editorial correction: AC-021.1 cited AC-002.3, which does not exist; it now cites AC-002.1. No change in meaning.</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="56" customWidth="1" min="2" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>ASR register (PED v3.0, ASR section)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>ASR</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Quality driver</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Source requirements and evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>ASR-01</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Ownership and status correctness under concurrent staff action</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>NFR-005; FR-011; FR-012; conflict C-1; RSK-009; RSK-010</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>ASR-02</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Authorisation and requester data privacy</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>NFR-003; NFR-006; FR-008; FR-014; FR-019; FR-020; RSK-011; RSK-012</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>ASR-03</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Auditability and tamper-evidence of controlled actions</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>NFR-007; FR-013; FR-022; RSK-013</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>ASR-04</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Oversight responsiveness and reporting that reconciles</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>NFR-004; NFR-008; FR-009; FR-015 to FR-018; FR-023; RSK-014</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>ASR-05</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Cost and complexity sustainability while staying ready to grow (restated, CR-011)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>NFR-009; conflicts C-4 and C-5; RSK-003; RSK-014; RSK-016</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>ASR-06</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Requester usability and timely status feedback</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>NFR-001; NFR-002; FR-001; FR-003; FR-007</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>ASR-07</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Growth readiness (new, CR-011)</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>NFR-010; conflict C-5; CR-010; CR-011</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>ADR index</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>ADR</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>ADR-001</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Architecture selection; continues D-001 and D-002</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>K. Marota</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Proposed, awaiting approval; to be revised under CR-010</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="25.5" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>ADR-002</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Persistence and data integrity: conditional update, append-only history, transaction boundaries</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>K. Marota</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Proposed, awaiting approval (uses A2 Task 2 research)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="25.5" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>ADR-003</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Technology stack with versions, licensing and security evidence; supersedes D-003</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>G. Enright</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Decision recorded 29/09/2026: .NET 10 LTS, ASP.NET Core, PostgreSQL 17.x. Awaiting approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>ADR-004</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Design decision 1: role-based view composition</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>M. Malope</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Proposed; revision 2 (08/10/2026) awaiting approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="25.5" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>ADR-005</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Design decision 2: RBAC policy and API security boundary; supersedes D-004</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>G. Enright</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Proposed, awaiting approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="25.5" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>ADR-006</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>API / integration decision: REST contract, validation, errors, versioning</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>K. Marota</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Proposed, awaiting approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>ADR-007</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Deployment direction, configuration and secrets</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>G. Enright</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>Decision recorded 29/09/2026: Render free tier, Neon free plan. Awaiting approval</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Map RTM rows to the ADR-001 services and add the FR-011 trace
Rewrites the RTM architecture, data and status columns so each requirement names its owning service and schema, with monolith code marked Changed (CR-010) until it moves into its service. Adds the FR-011 demonstration trace to the PED, following the app/ tree that CI builds and tests.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
@@ -653,12 +653,12 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Pages/Requests/Submit.cshtml (SubmitModel) -&gt; POST /api/v1/requests -&gt; RequestService -&gt; RequestRepository</t>
+          <t>FE submit page -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Request row created (unique reference, status Received); Category FK; required fields NOT NULL</t>
+          <t>requests schema: request row, ref ID, status Received; category ID checked through the ReferenceData API, no cross-schema FK</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q3" s="5" t="inlineStr">
@@ -740,12 +740,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>_CategorySelect partial on the submit page -&gt; GET /api/v1/categories -&gt; CategoryService -&gt; CategoryRepository</t>
+          <t>FE category select -&gt; entry -&gt; ReferenceData</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Category reference table; Request.category_id FK NOT NULL; retired categories kept for history</t>
+          <t>referencedata schema: category table, retired kept</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
@@ -827,12 +827,12 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Pages/Requests/Details.cshtml (DetailsModel) with the status badge tag helper -&gt; GET /api/v1/requests/{id}</t>
+          <t>FE status view -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Request.status read only; constrained status vocabulary, not free text</t>
+          <t>requests schema: constrained status, read-only to requesters</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q5" s="5" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Pages/Requests/Index.cshtml (IndexModel) -&gt; GET /api/v1/requests in own scope -&gt; AuthorisationPolicy</t>
+          <t>FE history -&gt; entry -&gt; Requests (scope from Access policy)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Query scoped by Request.requester_id; index on requester_id</t>
+          <t>requests schema: scoped by requester_id, indexed</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
@@ -1001,12 +1001,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>_FilterBar partial on Pages/Requests/Index.cshtml -&gt; GET /api/v1/requests with status filter</t>
+          <t>FE filter -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Composite index (requester_id, status); pagination</t>
+          <t>requests schema: (requester_id, status) index, paging</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
@@ -1088,12 +1088,12 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Not allocated while deferred</t>
+          <t>Not allocated (deferred)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Deliberately absent from the M2 schema; no Attachment entity or object storage</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>StatusTransitionService -&gt; FeedbackService -&gt; GET /api/v1/feedback -&gt; _FeedbackList partial on Pages/Requests/Index.cshtml</t>
+          <t>Requests writes feedback with the status change -&gt; entry -&gt; FE</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>FeedbackItem written in the same transaction as the status change; rejection reason mandatory</t>
+          <t>requests schema: feedback item in the same transaction as the status change</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
@@ -1262,12 +1262,12 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Queue.cshtml (QueueModel) with StaffQueueViewComponent -&gt; GET /api/v1/requests/queue -&gt; AuthorisationPolicy -&gt; RequestRepository</t>
+          <t>FE staff queue -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Rows filtered by role/team/assignment; composite index (status, category, assigned_to)</t>
+          <t>requests schema: queue indexes (status, category, assigned_to)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
@@ -1349,12 +1349,12 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>_FilterBar partial inside StaffQueueViewComponent -&gt; GET /api/v1/requests query parameters</t>
+          <t>FE queue filter and sort -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Indexes on status, category, created_at; sort whitelist; pagination</t>
+          <t>requests schema: indexes, sort whitelist, paging</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q11" s="5" t="inlineStr">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Details.cshtml (DetailsModel) with _RequestDetail and _HistoryList partials -&gt; GET /api/v1/requests/{id} -&gt; AuthorisationPolicy</t>
+          <t>FE staff detail -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Request joined to RequestStatusHistory and action notes; attachments absent (FR-006 deferred)</t>
+          <t>requests schema: request with history and notes</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Details.cshtml OnPostAcceptAsync -&gt; POST /api/v1/requests/{id}/assignment -&gt; AssignmentService -&gt; RequestRepository</t>
+          <t>FE accept -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>assigned_to + assigned_at; single-owner invariant by conditional UPDATE ... WHERE assigned_to IS NULL; history row appended</t>
+          <t>requests schema: conditional update where unassigned, history in the same transaction</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>In Development - M2 trace requirement</t>
+          <t>Changed (CR-010), M2 trace requirement</t>
         </is>
       </c>
       <c r="Q13" s="5" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Details.cshtml OnPostTransitionAsync -&gt; PATCH /api/v1/requests/{id}/status -&gt; StatusTransitionService</t>
+          <t>FE staff transition -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Status constrained; RequestStatusHistory append-only (actor, from, to, timestamp); validated inside the transaction</t>
+          <t>requests schema: guarded transitions, append-only history</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
@@ -1697,12 +1697,12 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Details.cshtml OnPostAddNoteAsync -&gt; POST /api/v1/requests/{id}/notes -&gt; HistoryRepository</t>
+          <t>FE staff note -&gt; entry -&gt; Requests</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Note rows append-only; no update or delete path exposed</t>
+          <t>requests schema: append-only notes</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="P15" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q15" s="5" t="inlineStr">
@@ -1784,12 +1784,12 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Details.cshtml OnPostCloseAsync -&gt; PATCH /api/v1/requests/{id}/status -&gt; AuthorisationPolicy, StatusTransitionService and FeedbackService</t>
+          <t>FE resolve or close -&gt; entry -&gt; Requests (close permission from Access policy)</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Resolution information stored; feedback row written in the same transaction</t>
+          <t>requests schema: resolution and feedback in the same transaction</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
@@ -1871,12 +1871,12 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Pages/Management/Oversight.cshtml with OversightTotalsViewComponent -&gt; GET /api/v1/reports/overview -&gt; ReportingService</t>
+          <t>FE oversight -&gt; entry -&gt; Reporting -&gt; Requests API</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Aggregates computed from the transactional tables; no separate reporting store (NFR-008)</t>
+          <t>No reporting copy; figures read through Requests (NFR-008)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -1958,12 +1958,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Pages/Management/Oversight.cshtml lifecycle filters -&gt; ReportingService</t>
+          <t>FE oversight filters -&gt; entry -&gt; Reporting -&gt; Requests API</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Requires a target_response_at field on Request - schema addition pending CR-005</t>
+          <t>Needs target_response_at in the requests schema (CR-005)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -2045,12 +2045,12 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>OversightTotalsViewComponent grouping -&gt; ReportingService</t>
+          <t>FE oversight grouping -&gt; entry -&gt; Reporting -&gt; Requests API</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Group-by on category and status with supporting indexes</t>
+          <t>No reporting copy; grouped through Requests</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -2132,12 +2132,12 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Pages/Management/Reports.cshtml (ReportsModel) -&gt; GET /api/v1/reports/performance -&gt; ReportingService</t>
+          <t>FE reports -&gt; entry -&gt; Reporting -&gt; Requests API</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Metrics derived from request and history tables; export scope pending CR-006</t>
+          <t>No reporting copy; export scope pending CR-006</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Pages/Admin/Users.cshtml (UsersModel) -&gt; /api/v1/admin/users -&gt; UserRoleService</t>
+          <t>FE admin users -&gt; entry -&gt; Access</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>User entity with active flag; deactivation blocks sign-in; no hard delete (audit retention)</t>
+          <t>access schema: users with active flag, no hard delete</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="P21" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q21" s="5" t="inlineStr">
@@ -2306,12 +2306,12 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Pages/Admin/Roles.cshtml (RolesModel) -&gt; /api/v1/admin/roles -&gt; AuthorisationPolicy as the single decision point</t>
+          <t>FE admin roles -&gt; entry -&gt; Access</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Role, Permission and UserRole tables; permission checks resolved server-side</t>
+          <t>access schema: roles, permissions, user roles</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
@@ -2393,12 +2393,12 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Pages/Admin/Categories.cshtml (CategoriesModel) -&gt; /api/v1/admin/categories -&gt; CategoryService</t>
+          <t>FE admin categories -&gt; entry -&gt; ReferenceData</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Category rows editable with retire flag; submission form reads the current list, no code change</t>
+          <t>referencedata schema: editable categories, retire flag</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -2480,12 +2480,12 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Pages/Admin/Audit.cshtml (AuditModel) -&gt; /api/v1/admin/audit -&gt; AuditService</t>
+          <t>FE admin audit -&gt; entry -&gt; Requests history, plus Access and ReferenceData change records</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Reads append-only history/audit tables; tamper-evident, no update path exposed</t>
+          <t>Append-only history in each owning schema</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
@@ -2567,12 +2567,12 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Reuse Pages/Management/Reports.cshtml at summary scope (access model pending CR-007)</t>
+          <t>FE summary reports -&gt; entry -&gt; Reporting -&gt; Requests API</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Same aggregates as FR-018 with a narrower scope; no additional entity</t>
+          <t>Same figures as FR-018 at summary scope</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
@@ -2654,12 +2654,12 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Pages/Requests/Submit.cshtml, one guided form with validation messages for each field</t>
+          <t>FE guided submit form</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>No schema impact</t>
+          <t>None</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
@@ -2741,12 +2741,12 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>FeedbackService write; JavaScript fetch polling refreshes the status partial on Pages/Requests/Details.cshtml</t>
+          <t>Requests -&gt; entry -&gt; FE polling</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>FeedbackItem written in the same transaction as the status change</t>
+          <t>requests schema: feedback in the same transaction</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>AuthorisationPolicy with ownership scoped repository queries in every page model</t>
+          <t>Access policy, checked again in every service</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>requester_id scoping on every request read; no unscoped read path</t>
+          <t>requests schema: requester_id scoping on every read</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Queue and oversight query paths: StaffQueueViewComponent, RequestRepository, ReportingService</t>
+          <t>Queue in Requests, oversight in Reporting</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Indexing and pagination; aggregates read from the same store</t>
+          <t>requests schema: indexes and paging</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -3002,12 +3002,12 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>AssignmentService and StatusTransitionService behind the API boundary</t>
+          <t>Requests only</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Conditional update / optimistic concurrency; single-owner invariant enforced at database level</t>
+          <t>requests schema: conditional updates, single-owner check</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>In Development - M2 trace requirement</t>
+          <t>Changed (CR-010), M2 trace requirement</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -3089,12 +3089,12 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>AuthorisationPolicy invoked by every page handler and every endpoint</t>
+          <t>Access policy, checked again in every service</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Role and permission tables; checks never rely on UI state</t>
+          <t>access schema: role and permission rules</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
@@ -3176,12 +3176,12 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>AuditService and append only history writes on every controlled action</t>
+          <t>Requests only, plus change records in Access and ReferenceData</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Append-only tables; no UPDATE or DELETE endpoints over history rows</t>
+          <t>Append-only history in each owning schema</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>In Development</t>
+          <t>Changed (CR-010)</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
@@ -3263,12 +3263,12 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>ReportingService reading the transactional tables</t>
+          <t>Reporting reads through Requests</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Aggregates computed from source tables; no duplicated store to drift</t>
+          <t>No duplicated store</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
@@ -3350,12 +3350,12 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Whole solution deployed as a single deployable unit</t>
+          <t>Four services, entry point and FE on free tiers</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>One managed PostgreSQL instance on a free or low-cost tier; backup limits recorded</t>
+          <t>One shared PostgreSQL instance, schema per service</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -3437,12 +3437,12 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Pending revised ADR-001 (CR-010)</t>
+          <t>All services</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>Each service owns its data store; pending revised ADR-001/ADR-002 (CR-010)</t>
+          <t>Schema per service, no cross-schema access</t>
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Mark RTM verification evidence by whether it runs in CI
Rewrites the RTM verification column to separate tests that run in the CI Quality Gate from Backend/ tests that never run there, and adds a short verification-evidence note to the PED. Only StatusTransitionTests and AssignmentServiceTests currently count as CI evidence; ConcurrentAcceptTests is skipped until CI has a test database.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v2.0.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="N3" s="5" t="inlineStr">
         <is>
-          <t>RequestServiceTests (Overlong_title_is_refused, Staff_cannot_submit_requests_without_the_permission); not yet executed</t>
+          <t>Not in CI: Backend RequestServiceTests (Overlong_title_is_refused, Staff_cannot_submit_requests_without_the_permission). Planned in CI</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>Covered indirectly by RequestServiceTests; page test planned</t>
+          <t>Not in CI: covered indirectly by Backend RequestServiceTests. Planned: category test in CI</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>StatusRulesTests (Display_text_is_plain_language); page test for AC-003.2 planned</t>
+          <t>Not in CI: Backend StatusRulesTests (Display_text_is_plain_language). Planned: page test for AC-003.2</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>RequestServiceTests scope cases; negative access test planned</t>
+          <t>Not in CI: Backend RequestServiceTests scope cases. Planned: negative access test</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>NoteAndFeedbackTests (Nobody_can_mark_someone_elses_feedback_as_read); timing check planned</t>
+          <t>Not in CI: Backend NoteAndFeedbackTests (Nobody_can_mark_someone_elses_feedback_as_read). Planned: timing check</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>RequestServiceTests (The_queue_is_closed_to_requesters); not yet executed</t>
+          <t>Not in CI: Backend RequestServiceTests (The_queue_is_closed_to_requesters). Planned in CI</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>RequestServiceTests visibility cases; not yet executed</t>
+          <t>Not in CI: Backend RequestServiceTests visibility cases. Planned in CI</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>RealDatabaseTests.Ten_staff_accepting_at_once_leaves_exactly_one_owner (TC-011.2) and AssignmentServiceTests; needs a test database, not yet executed</t>
+          <t>CI: AssignmentServiceTests (4 cases, run in the gate); ConcurrentAcceptTests skipped in CI until a test database is provided. Not in CI: Backend RealDatabaseTests</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>StatusTransitionServiceTests (7 cases) and StatusRulesTests; not yet executed</t>
+          <t>CI: StatusTransitionTests (4 allowed, 4 refused transitions). Not in CI: Backend StatusTransitionServiceTests and StatusRulesTests</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>NoteAndFeedbackTests (Only_the_owner_can_add_notes, An_empty_note_is_refused)</t>
+          <t>Not in CI: Backend NoteAndFeedbackTests (Only_the_owner_can_add_notes, An_empty_note_is_refused). Planned in CI</t>
         </is>
       </c>
       <c r="O15" s="6" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>StatusTransitionServiceTests close cases; not yet executed</t>
+          <t>Not in CI: Backend StatusTransitionServiceTests close cases. Planned in CI</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>RequestServiceTests and AssignmentServiceTests permission cases (A_requester_cannot_accept_requests, A_requester_cannot_change_status)</t>
+          <t>CI: AssignmentServiceTests (The_policy_is_checked_before_anything_is_written). Not in CI: Backend permission cases</t>
         </is>
       </c>
       <c r="O22" s="6" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="N24" s="6" t="inlineStr">
         <is>
-          <t>RealDatabaseTests.History_rows_cannot_be_changed_or_deleted</t>
+          <t>Not in CI: Backend RealDatabaseTests (History_rows_cannot_be_changed_or_deleted). Planned in CI</t>
         </is>
       </c>
       <c r="O24" s="6" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>RequestServiceTests visibility cases; direct reference negative test planned</t>
+          <t>Not in CI: Backend RequestServiceTests visibility cases. Planned: direct reference negative test</t>
         </is>
       </c>
       <c r="O28" s="6" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>RealDatabaseTests.Ten_staff_accepting_at_once_leaves_exactly_one_owner and The_database_itself_refuses_an_owner_on_a_Received_request</t>
+          <t>CI: AssignmentServiceTests; ConcurrentAcceptTests skipped in CI until a test database is provided. Not in CI: Backend RealDatabaseTests</t>
         </is>
       </c>
       <c r="O30" s="6" t="inlineStr">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="N31" s="5" t="inlineStr">
         <is>
-          <t>Permission refusal cases across the service tests; role matrix test planned</t>
+          <t>CI: AssignmentServiceTests policy check. Not in CI: Backend permission cases. Planned: role matrix test</t>
         </is>
       </c>
       <c r="O31" s="6" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>RealDatabaseTests.History_rows_cannot_be_changed_or_deleted</t>
+          <t>Not in CI: Backend RealDatabaseTests (History_rows_cannot_be_changed_or_deleted). Planned in CI</t>
         </is>
       </c>
       <c r="O32" s="6" t="inlineStr">

</xml_diff>